<commit_message>
Save local work before pull
</commit_message>
<xml_diff>
--- a/data/nba_injuries.xlsx
+++ b/data/nba_injuries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\letsparlayml.github.io\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CC917F2-3FCC-49B5-9F48-FC4A28F7A4D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A0BA91-9673-45F0-AA69-4218EA163E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="88">
   <si>
     <t>NBA Injury Context Template</t>
   </si>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>Luka Doncic</t>
+  </si>
+  <si>
+    <t>Moses Moody</t>
   </si>
 </sst>
 </file>
@@ -795,7 +798,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1618,6 +1621,20 @@
         <v>28</v>
       </c>
       <c r="D50" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A51" s="9">
+        <v>46108</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D51" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update site scripts and data
</commit_message>
<xml_diff>
--- a/data/nba_injuries.xlsx
+++ b/data/nba_injuries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\letsparlayml.github.io\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6898AFD3-47DC-4188-BFEF-237789A01C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BE1D3A-36A0-408D-97D1-A802572B9E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,14 +18,14 @@
     <sheet name="status_reference" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">injuries_input!$A$1:$G$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">injuries_input!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="94">
   <si>
     <t>NBA Injury Context Template</t>
   </si>
@@ -96,18 +96,6 @@
     <t>Quick rules</t>
   </si>
   <si>
-    <t>CLE</t>
-  </si>
-  <si>
-    <t>Jaylon Tyson</t>
-  </si>
-  <si>
-    <t>Jarrett Allen</t>
-  </si>
-  <si>
-    <t>Craig Porter</t>
-  </si>
-  <si>
     <t>IND</t>
   </si>
   <si>
@@ -117,54 +105,15 @@
     <t>Obi Toppin</t>
   </si>
   <si>
-    <t>Isaac Okoro</t>
-  </si>
-  <si>
-    <t>CHI</t>
-  </si>
-  <si>
-    <t>Anfernee Simons</t>
-  </si>
-  <si>
-    <t>Guershchon Yabusele</t>
-  </si>
-  <si>
     <t>Nikola Vucevic</t>
   </si>
   <si>
     <t>BOS</t>
   </si>
   <si>
-    <t>Ty Jerome</t>
-  </si>
-  <si>
-    <t>MEM</t>
-  </si>
-  <si>
-    <t>Jaylen Wells</t>
-  </si>
-  <si>
-    <t>Jahmai Mashack</t>
-  </si>
-  <si>
-    <t>UTA</t>
-  </si>
-  <si>
-    <t>Isaiah Collier</t>
-  </si>
-  <si>
-    <t>Keyonte George</t>
-  </si>
-  <si>
-    <t>Lauri Markkanen</t>
-  </si>
-  <si>
     <t>LAC</t>
   </si>
   <si>
-    <t>Jordan Miller</t>
-  </si>
-  <si>
     <t>Jaylen Brown</t>
   </si>
   <si>
@@ -174,21 +123,9 @@
     <t>Derrick White</t>
   </si>
   <si>
-    <t>Jaime Jaquez</t>
-  </si>
-  <si>
     <t>MIA</t>
   </si>
   <si>
-    <t>Dean Wade</t>
-  </si>
-  <si>
-    <t>Rob Dillingham</t>
-  </si>
-  <si>
-    <t>Nick Richards</t>
-  </si>
-  <si>
     <t>Gary Harris</t>
   </si>
   <si>
@@ -201,103 +138,175 @@
     <t>Bobby Portis</t>
   </si>
   <si>
-    <t>Myles Turner</t>
-  </si>
-  <si>
     <t>Giannis Antetokounmpo</t>
   </si>
   <si>
     <t>Kevin Porter Jr.</t>
   </si>
   <si>
-    <t>Caris LeVert</t>
-  </si>
-  <si>
-    <t>DET</t>
-  </si>
-  <si>
-    <t>Marcus Sasser</t>
-  </si>
-  <si>
-    <t>Jalen Duren</t>
-  </si>
-  <si>
-    <t>Tobias Harris</t>
-  </si>
-  <si>
-    <t>Duncan Robinson</t>
-  </si>
-  <si>
-    <t>Ausar Thompson</t>
-  </si>
-  <si>
-    <t>Cade Cunningham</t>
-  </si>
-  <si>
-    <t>Isaiah Stewart</t>
-  </si>
-  <si>
-    <t>Ayo Dosunmu</t>
-  </si>
-  <si>
-    <t>MIN</t>
-  </si>
-  <si>
-    <t>Anthony Edwards</t>
-  </si>
-  <si>
-    <t>Jaden McDaniels</t>
-  </si>
-  <si>
-    <t>Tyrese Maxey</t>
-  </si>
-  <si>
-    <t>PHI</t>
-  </si>
-  <si>
-    <t>Kelly Oubre Jr.</t>
-  </si>
-  <si>
-    <t>Johni Broome</t>
-  </si>
-  <si>
     <t>Tidjane Salaun</t>
   </si>
   <si>
-    <t>Nique Clifford</t>
-  </si>
-  <si>
     <t>SAC</t>
   </si>
   <si>
-    <t>Killian Hayes</t>
-  </si>
-  <si>
     <t>Keegan Murray</t>
   </si>
   <si>
     <t>Russell Westbrook</t>
   </si>
   <si>
-    <t>Jock Landale</t>
-  </si>
-  <si>
-    <t>ATL</t>
-  </si>
-  <si>
-    <t>Dillon Brooks</t>
-  </si>
-  <si>
-    <t>PHX</t>
-  </si>
-  <si>
-    <t>Amir Coffey</t>
-  </si>
-  <si>
-    <t>Haywood Highsmith</t>
-  </si>
-  <si>
-    <t>Mark Williams</t>
+    <t>Isaiah Jackson</t>
+  </si>
+  <si>
+    <t>Thanasis Antetokounmpo</t>
+  </si>
+  <si>
+    <t>Norman Powell</t>
+  </si>
+  <si>
+    <t>TJ McConnell</t>
+  </si>
+  <si>
+    <t>Andrew Nembhard</t>
+  </si>
+  <si>
+    <t>Pascal Siakam</t>
+  </si>
+  <si>
+    <t>Jarace Walker</t>
+  </si>
+  <si>
+    <t>Isaiah Stevens</t>
+  </si>
+  <si>
+    <t>Josh Minott</t>
+  </si>
+  <si>
+    <t>BKN</t>
+  </si>
+  <si>
+    <t>Michael Porter Jr.</t>
+  </si>
+  <si>
+    <t>Danny Wolf</t>
+  </si>
+  <si>
+    <t>Leaky Black</t>
+  </si>
+  <si>
+    <t>WAS</t>
+  </si>
+  <si>
+    <t>Bilal Coulibaly</t>
+  </si>
+  <si>
+    <t>Anthony Davis</t>
+  </si>
+  <si>
+    <t>Kyshawn George</t>
+  </si>
+  <si>
+    <t>Tre Johnson</t>
+  </si>
+  <si>
+    <t>Alex Sarr</t>
+  </si>
+  <si>
+    <t>Trae Young</t>
+  </si>
+  <si>
+    <t>Robert Williams</t>
+  </si>
+  <si>
+    <t>POR</t>
+  </si>
+  <si>
+    <t>Jerami Grant</t>
+  </si>
+  <si>
+    <t>Vit Krejci</t>
+  </si>
+  <si>
+    <t>Shaedon Sharpe</t>
+  </si>
+  <si>
+    <t>Anthony Black</t>
+  </si>
+  <si>
+    <t>ORL</t>
+  </si>
+  <si>
+    <t>Jonathan Issac</t>
+  </si>
+  <si>
+    <t>Franz Wagner</t>
+  </si>
+  <si>
+    <t>Brandon Ingram</t>
+  </si>
+  <si>
+    <t>TOR</t>
+  </si>
+  <si>
+    <t>Trayce Jackson-Davis</t>
+  </si>
+  <si>
+    <t>Collin Murray-Boyles</t>
+  </si>
+  <si>
+    <t>Chucky Hepburn</t>
+  </si>
+  <si>
+    <t>Immanual Quickley</t>
+  </si>
+  <si>
+    <t>Jayson Tatum</t>
+  </si>
+  <si>
+    <t>CHA</t>
+  </si>
+  <si>
+    <t>Trey Murphy III</t>
+  </si>
+  <si>
+    <t>NOP</t>
+  </si>
+  <si>
+    <t>Dejounte Murray</t>
+  </si>
+  <si>
+    <t>Bryce McGowens</t>
+  </si>
+  <si>
+    <t>Kevin McCullar</t>
+  </si>
+  <si>
+    <t>NYK</t>
+  </si>
+  <si>
+    <t>Miles McBride</t>
+  </si>
+  <si>
+    <t>Landry Shamet</t>
+  </si>
+  <si>
+    <t>Seth Curry</t>
+  </si>
+  <si>
+    <t>GSW</t>
+  </si>
+  <si>
+    <t>Quinten Post</t>
+  </si>
+  <si>
+    <t>Will Richard</t>
+  </si>
+  <si>
+    <t>Stephen Curry</t>
+  </si>
+  <si>
+    <t>Al Horford</t>
   </si>
 </sst>
 </file>
@@ -847,177 +856,147 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+        <v>34</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>24</v>
@@ -1025,309 +1004,285 @@
       <c r="C12" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
+        <v>23</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+        <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="9">
-        <v>46108</v>
+        <v>46110</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A20" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A17" s="9">
-        <v>46108</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A18" s="9">
-        <v>46108</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A19" s="9">
-        <v>46108</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A20" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B20" s="7" t="s">
+      <c r="C20" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A21" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C21" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A22" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A21" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B21" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A22" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B22" s="7" t="s">
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A23" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A23" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A24" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C23" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A24" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B24" s="7" t="s">
+      <c r="C24" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D24" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A25" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A26" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A26" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B26" s="7" t="s">
+      <c r="C26" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D26" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A27" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C27" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A28" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B28" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D26" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A27" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B27" s="6" t="s">
+      <c r="C28" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A29" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D27" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A28" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B28" s="7" t="s">
+      <c r="C29" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="D28" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A29" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B29" s="6" t="s">
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A30" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B30" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D29" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A30" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B30" s="7" t="s">
+      <c r="C30" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A31" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="D30" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A31" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A32" s="9">
+        <v>46110</v>
+      </c>
+      <c r="B32" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A32" s="9">
-        <v>46109</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>68</v>
-      </c>
       <c r="C32" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D32" t="s">
         <v>14</v>
@@ -1335,13 +1290,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B33" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="D33" t="s">
         <v>14</v>
@@ -1349,27 +1304,27 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>70</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
         <v>14</v>
@@ -1377,27 +1332,27 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C36" s="7" t="s">
-        <v>71</v>
-      </c>
       <c r="D36" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>74</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
@@ -1405,13 +1360,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
@@ -1419,13 +1374,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D39" t="s">
         <v>14</v>
@@ -1433,13 +1388,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>31</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
         <v>14</v>
@@ -1447,13 +1402,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
@@ -1461,13 +1416,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
@@ -1475,69 +1430,69 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A43" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="D43" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="D44" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="D45" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A46" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="D46" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A47" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>31</v>
+        <v>81</v>
       </c>
       <c r="D47" t="s">
         <v>11</v>
@@ -1545,13 +1500,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A48" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
@@ -1559,27 +1514,27 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A49" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="D49" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A50" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>37</v>
+        <v>85</v>
       </c>
       <c r="D50" t="s">
         <v>11</v>
@@ -1587,83 +1542,83 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A51" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="D51" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A52" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="D52" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A53" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="D53" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A54" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D54" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A55" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D55" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A56" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B56" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C56" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>87</v>
       </c>
       <c r="D56" t="s">
         <v>14</v>
@@ -1671,20 +1626,20 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A57" s="9">
-        <v>46109</v>
+        <v>46110</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D57" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G53" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:G1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1693,7 +1648,7 @@
           <x14:formula1>
             <xm:f>status_reference!$A$2:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D353</xm:sqref>
+          <xm:sqref>D2:D297</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Daily live site update
</commit_message>
<xml_diff>
--- a/data/nba_injuries.xlsx
+++ b/data/nba_injuries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\letsparlayml.github.io\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24FF0B88-0526-409E-8572-7F02D6B7DA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8CFFB5-8BAE-4117-A439-E74D4E9CB493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
   <si>
     <t>NBA Injury Context Template</t>
   </si>
@@ -96,28 +96,37 @@
     <t>Quick rules</t>
   </si>
   <si>
-    <t>MIA</t>
-  </si>
-  <si>
-    <t>Dru Smith</t>
-  </si>
-  <si>
-    <t>Nikola Jovic</t>
-  </si>
-  <si>
-    <t>POR</t>
-  </si>
-  <si>
-    <t>Jerami Grant</t>
-  </si>
-  <si>
-    <t>PHX</t>
-  </si>
-  <si>
-    <t>Grayson Allen</t>
-  </si>
-  <si>
-    <t>Pelle Larsson</t>
+    <t>Jett Howard</t>
+  </si>
+  <si>
+    <t>ORL</t>
+  </si>
+  <si>
+    <t>Jonathan Isaac</t>
+  </si>
+  <si>
+    <t>Trent Watford</t>
+  </si>
+  <si>
+    <t>PHI</t>
+  </si>
+  <si>
+    <t>Johni Broome</t>
+  </si>
+  <si>
+    <t>Joel Embiid</t>
+  </si>
+  <si>
+    <t>Quinten Post</t>
+  </si>
+  <si>
+    <t>GSW</t>
+  </si>
+  <si>
+    <t>Isaiah Jackson</t>
+  </si>
+  <si>
+    <t>LAC</t>
   </si>
 </sst>
 </file>
@@ -217,9 +226,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,15 +540,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.65">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="3" spans="1:7" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
@@ -623,7 +632,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -662,72 +671,100 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A2" s="9">
-        <v>46126</v>
+      <c r="A2" s="7">
+        <v>46127</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A3" s="9">
-        <v>46126</v>
+      <c r="A3" s="7">
+        <v>46127</v>
       </c>
       <c r="B3" t="s">
         <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A4" s="7">
+        <v>46127</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A5" s="7">
+        <v>46127</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A4" s="9">
-        <v>46126</v>
-      </c>
-      <c r="B4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A5" s="9">
-        <v>46126</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-    </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A6" s="9">
-        <v>46126</v>
+      <c r="A6" s="7">
+        <v>46127</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A7" s="7">
+        <v>46127</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A8" s="7">
+        <v>46127</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>